<commit_message>
added g17 batch testing file
</commit_message>
<xml_diff>
--- a/Tests/g17_setup1_with_1ed_sim_outputs.xlsx
+++ b/Tests/g17_setup1_with_1ed_sim_outputs.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -426,10 +426,10 @@
         <v>3</v>
       </c>
       <c r="D1" t="n">
-        <v>3600000</v>
+        <v>10000</v>
       </c>
       <c r="E1" t="n">
-        <v>3</v>
+        <v>1000</v>
       </c>
       <c r="F1" t="inlineStr">
         <is>
@@ -445,7 +445,7 @@
         </is>
       </c>
       <c r="I1" t="n">
-        <v>3098.856206443471</v>
+        <v>3160.296349178773</v>
       </c>
       <c r="J1" t="inlineStr">
         <is>
@@ -453,7 +453,7 @@
         </is>
       </c>
       <c r="K1" t="n">
-        <v>3068.145626459736</v>
+        <v>59.02441188320518</v>
       </c>
       <c r="L1" t="inlineStr">
         <is>
@@ -461,7 +461,7 @@
         </is>
       </c>
       <c r="M1" t="n">
-        <v>3130.423959321342</v>
+        <v>27250.68447063304</v>
       </c>
     </row>
     <row r="2">
@@ -475,10 +475,10 @@
         <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>3600000</v>
+        <v>20000</v>
       </c>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>1000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>2898.552358993019</v>
+        <v>3316.064824346746</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>2841.942546507344</v>
+        <v>56.87332554720342</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -510,7 +510,7 @@
         </is>
       </c>
       <c r="M2" t="n">
-        <v>2948.509186495095</v>
+        <v>29970.00729409792</v>
       </c>
     </row>
     <row r="3">
@@ -524,10 +524,10 @@
         <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>3600000</v>
+        <v>30000</v>
       </c>
       <c r="E3" t="n">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -543,7 +543,7 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>3092.159048875361</v>
+        <v>3428.92615750902</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -551,7 +551,7 @@
         </is>
       </c>
       <c r="K3" t="n">
-        <v>2806.137142042164</v>
+        <v>60.19994493946433</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
@@ -559,7 +559,7 @@
         </is>
       </c>
       <c r="M3" t="n">
-        <v>4001.014171928167</v>
+        <v>24808.61110525485</v>
       </c>
     </row>
     <row r="4">
@@ -573,10 +573,10 @@
         <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>3600000</v>
+        <v>40000</v>
       </c>
       <c r="E4" t="n">
-        <v>100</v>
+        <v>1000</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -592,7 +592,7 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>3161.447240878717</v>
+        <v>3182.366199608689</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -600,7 +600,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>2441.128696590662</v>
+        <v>57.41541673615575</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
@@ -608,7 +608,105 @@
         </is>
       </c>
       <c r="M4" t="n">
-        <v>3721.377990454435</v>
+        <v>20238.89758048207</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" t="n">
+        <v>50000</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>3040.721233797079</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>63.5209624543786</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>20794.12405123189</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" t="n">
+        <v>60000</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>3135.924618098682</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>52.54934802278876</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>20101.71023960784</v>
       </c>
     </row>
   </sheetData>

</xml_diff>